<commit_message>
added the big five files and female1 headshot data
</commit_message>
<xml_diff>
--- a/Models/CLIP/female1/clip_trait_similarities_female1.xlsx
+++ b/Models/CLIP/female1/clip_trait_similarities_female1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tamucs-my.sharepoint.com/personal/yq_c_tamu_edu/Documents/Research/genderBias/GenderBias-SRL-Implementation/Models/CLIP/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tamucs-my.sharepoint.com/personal/yq_c_tamu_edu/Documents/Research/genderBias/GenderBias-SRL-Implementation/Models/CLIP/female1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="11_2B59D2BFD340DD7A6864B1335B1510344D07F15D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{255E19AE-6330-4C6E-91CD-BBC06A8EAB35}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="11_2B59D2BFD340DD7A6864B1335B1510344D07F15D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67185978-2EC0-40C0-8FF9-AE7C32E9B6E2}"/>
   <bookViews>
-    <workbookView xWindow="2620" yWindow="120" windowWidth="11820" windowHeight="10890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Negative Trait</t>
   </si>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>avg</t>
+  </si>
+  <si>
+    <t>difference (pos-neg)</t>
   </si>
 </sst>
 </file>
@@ -436,16 +439,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.26953125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -458,8 +462,11 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -472,8 +479,12 @@
       <c r="D2">
         <v>1.2468745931982991E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E2">
+        <f>D2-B2</f>
+        <v>1.17317028343677E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -486,8 +497,12 @@
       <c r="D3">
         <v>8.5168935358524323E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E3">
+        <f t="shared" ref="E3:E7" si="0">D3-B3</f>
+        <v>-1.2991614639759064E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -500,8 +515,12 @@
       <c r="D4">
         <v>0.2870514988899231</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>0.23420187830924988</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -514,8 +533,12 @@
       <c r="D5">
         <v>3.601866215467453E-2</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>-2.9046274721622467E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -528,8 +551,12 @@
       <c r="D6">
         <v>0.1068233251571655</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>5.8195002377033213E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -542,8 +569,12 @@
       <c r="D7">
         <v>0.1427941620349884</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>8.911842480301857E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>

</xml_diff>